<commit_message>
everything updated. code comments removed partially, and new scripts made more effecient. also large amounts of paper cuts where not truly helpful, including rremoving top-02 and rmse/mae ratio.
</commit_message>
<xml_diff>
--- a/Analysis/Sensitivity_merec_entropy_arms_deepseek.xlsx
+++ b/Analysis/Sensitivity_merec_entropy_arms_deepseek.xlsx
@@ -961,7 +961,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>{"HVAC": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Appliance": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Shower": {"energy_cost": 0.248, "environmental": 0.244, "comfort": 0.203, "practicality": 0.305}}</t>
+          <t>{"HVAC": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Appliance": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Shower": {"energy_cost": 0.251251, "environmental": 0.245245, "comfort": 0.203203, "practicality": 0.3003}}</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -970,22 +970,22 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.09372</v>
+        <v>0.09301999999999999</v>
       </c>
       <c r="F14" t="n">
-        <v>0.09409999999999999</v>
+        <v>0.09408000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>0.3369</v>
+        <v>0.3338</v>
       </c>
       <c r="H14" t="n">
-        <v>0.6932</v>
+        <v>0.6953</v>
       </c>
       <c r="I14" t="n">
-        <v>0.14664</v>
+        <v>0.14254</v>
       </c>
       <c r="J14" t="n">
-        <v>0.89254</v>
+        <v>0.8939</v>
       </c>
     </row>
     <row r="15">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>{"HVAC": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Appliance": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Shower": {"energy_cost": 0.248, "environmental": 0.244, "comfort": 0.203, "practicality": 0.305}}</t>
+          <t>{"HVAC": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Appliance": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Shower": {"energy_cost": 0.251251, "environmental": 0.245245, "comfort": 0.203203, "practicality": 0.3003}}</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1010,22 +1010,22 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.24036</v>
+        <v>0.23556</v>
       </c>
       <c r="F15" t="n">
-        <v>0.26206</v>
+        <v>0.25692</v>
       </c>
       <c r="G15" t="n">
-        <v>0.49026</v>
+        <v>0.4800000000000001</v>
       </c>
       <c r="H15" t="n">
-        <v>0.78976</v>
+        <v>0.78872</v>
       </c>
       <c r="I15" t="n">
-        <v>0.14664</v>
+        <v>0.14254</v>
       </c>
       <c r="J15" t="n">
-        <v>0.89254</v>
+        <v>0.8939</v>
       </c>
     </row>
     <row r="16">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>{"HVAC": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Appliance": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Shower": {"energy_cost": 0.248, "environmental": 0.244, "comfort": 0.203, "practicality": 0.305}}</t>
+          <t>{"HVAC": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Appliance": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Shower": {"energy_cost": 0.251251, "environmental": 0.245245, "comfort": 0.203203, "practicality": 0.3003}}</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1050,22 +1050,22 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.89254</v>
+        <v>0.8939</v>
       </c>
       <c r="F16" t="n">
-        <v>0.9111799999999999</v>
+        <v>0.9117</v>
       </c>
       <c r="G16" t="n">
-        <v>0.9096399999999999</v>
+        <v>0.9116799999999999</v>
       </c>
       <c r="H16" t="n">
         <v>0.9887</v>
       </c>
       <c r="I16" t="n">
-        <v>0.14664</v>
+        <v>0.14254</v>
       </c>
       <c r="J16" t="n">
-        <v>0.89254</v>
+        <v>0.8939</v>
       </c>
     </row>
     <row r="17">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>{"HVAC": {"energy_cost": 0.336336, "environmental": 0.32032, "comfort": 0.269269, "practicality": 0.074074}, "Appliance": {"energy_cost": 0.193, "environmental": 0.465, "comfort": 0.124, "practicality": 0.218}, "Shower": {"energy_cost": 0.333666, "environmental": 0.313686, "comfort": 0.126873, "practicality": 0.225774}}</t>
+          <t>{"HVAC": {"energy_cost": 0.336336, "environmental": 0.32032, "comfort": 0.269269, "practicality": 0.074074}, "Appliance": {"energy_cost": 0.193, "environmental": 0.465, "comfort": 0.124, "practicality": 0.218}, "Shower": {"energy_cost": 0.335, "environmental": 0.316, "comfort": 0.122, "practicality": 0.227}}</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1090,22 +1090,22 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.08821999999999999</v>
+        <v>0.09029999999999999</v>
       </c>
       <c r="F17" t="n">
-        <v>0.08734</v>
+        <v>0.08890000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>0.342</v>
+        <v>0.34612</v>
       </c>
       <c r="H17" t="n">
-        <v>0.70766</v>
+        <v>0.70662</v>
       </c>
       <c r="I17" t="n">
-        <v>0.25878</v>
+        <v>0.2594400000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>0.8959400000000001</v>
+        <v>0.90144</v>
       </c>
     </row>
     <row r="18">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>{"HVAC": {"energy_cost": 0.336336, "environmental": 0.32032, "comfort": 0.269269, "practicality": 0.074074}, "Appliance": {"energy_cost": 0.193, "environmental": 0.465, "comfort": 0.124, "practicality": 0.218}, "Shower": {"energy_cost": 0.333666, "environmental": 0.313686, "comfort": 0.126873, "practicality": 0.225774}}</t>
+          <t>{"HVAC": {"energy_cost": 0.336336, "environmental": 0.32032, "comfort": 0.269269, "practicality": 0.074074}, "Appliance": {"energy_cost": 0.193, "environmental": 0.465, "comfort": 0.124, "practicality": 0.218}, "Shower": {"energy_cost": 0.335, "environmental": 0.316, "comfort": 0.122, "practicality": 0.227}}</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1130,22 +1130,22 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.347</v>
+        <v>0.3497400000000001</v>
       </c>
       <c r="F18" t="n">
-        <v>0.36874</v>
+        <v>0.3718</v>
       </c>
       <c r="G18" t="n">
-        <v>0.5599999999999999</v>
+        <v>0.56206</v>
       </c>
       <c r="H18" t="n">
-        <v>0.8297399999999999</v>
+        <v>0.8328199999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>0.25878</v>
+        <v>0.2594400000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>0.8959400000000001</v>
+        <v>0.90144</v>
       </c>
     </row>
     <row r="19">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>{"HVAC": {"energy_cost": 0.336336, "environmental": 0.32032, "comfort": 0.269269, "practicality": 0.074074}, "Appliance": {"energy_cost": 0.193, "environmental": 0.465, "comfort": 0.124, "practicality": 0.218}, "Shower": {"energy_cost": 0.333666, "environmental": 0.313686, "comfort": 0.126873, "practicality": 0.225774}}</t>
+          <t>{"HVAC": {"energy_cost": 0.336336, "environmental": 0.32032, "comfort": 0.269269, "practicality": 0.074074}, "Appliance": {"energy_cost": 0.193, "environmental": 0.465, "comfort": 0.124, "practicality": 0.218}, "Shower": {"energy_cost": 0.335, "environmental": 0.316, "comfort": 0.122, "practicality": 0.227}}</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1170,22 +1170,22 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.8959400000000001</v>
+        <v>0.90144</v>
       </c>
       <c r="F19" t="n">
-        <v>0.9106799999999999</v>
+        <v>0.91476</v>
       </c>
       <c r="G19" t="n">
-        <v>0.924</v>
+        <v>0.9322199999999998</v>
       </c>
       <c r="H19" t="n">
         <v>0.98766</v>
       </c>
       <c r="I19" t="n">
-        <v>0.25878</v>
+        <v>0.2594400000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>0.8959400000000001</v>
+        <v>0.90144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>